<commit_message>
Added more details in initial few chapters
</commit_message>
<xml_diff>
--- a/MSE_motivation.xlsx
+++ b/MSE_motivation.xlsx
@@ -1,37 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tiss-2025\learning-isl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC821F29-3802-48A2-B7D7-7A250CE80893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB60C23-E3F1-4D11-A00E-A34D52062062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{8519553A-6E39-4723-8F51-C21798431B9A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8519553A-6E39-4723-8F51-C21798431B9A}"/>
   </bookViews>
   <sheets>
     <sheet name="MSE_1" sheetId="1" r:id="rId1"/>
     <sheet name="MSE_2" sheetId="2" r:id="rId2"/>
     <sheet name="Accuracy" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>